<commit_message>
Actualización BIM Wed Apr  8 21:47:39 UTC 2026
</commit_message>
<xml_diff>
--- a/data/bim_normativas.xlsx
+++ b/data/bim_normativas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,6 +469,11 @@
           <t>fuente</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>timestamp</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -510,6 +515,9 @@
         <is>
           <t>https://example.com</t>
         </is>
+      </c>
+      <c r="I2" t="n">
+        <v>1775684859.319966</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización BIM Wed Apr  8 22:01:11 UTC 2026
</commit_message>
<xml_diff>
--- a/data/bim_normativas.xlsx
+++ b/data/bim_normativas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,16 +469,11 @@
           <t>fuente</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>timestamp</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Normativa BIM Test</t>
+          <t>TEST BIM</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -493,12 +488,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2024-01-01</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2024-02-01</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -513,11 +508,8 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://example.com</t>
-        </is>
-      </c>
-      <c r="I2" t="n">
-        <v>1775684859.319966</v>
+          <t>https://test.com</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización BIM Wed Apr  8 22:07:51 UTC 2026
</commit_message>
<xml_diff>
--- a/data/bim_normativas.xlsx
+++ b/data/bim_normativas.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,42 +417,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>nombre</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>pais</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>region</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>fecha_publicacion</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>entrada_vigor</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>estado</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>fuente</t>
         </is>

</xml_diff>

<commit_message>
Actualización BIM Wed Apr  8 22:11:32 UTC 2026
</commit_message>
<xml_diff>
--- a/data/bim_normativas.xlsx
+++ b/data/bim_normativas.xlsx
@@ -476,12 +476,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024-01-01</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024-02-01</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">

</xml_diff>

<commit_message>
Actualización BIM Wed Apr  8 22:30:34 UTC 2026
</commit_message>
<xml_diff>
--- a/data/bim_normativas.xlsx
+++ b/data/bim_normativas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,42 +461,342 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TEST BIM</t>
+          <t>Bim Afolami MP</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>España</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Madrid</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2024-01-01</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2024-02-01</t>
-        </is>
-      </c>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>detectado</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>vigente</t>
+          <t>pendiente validación</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://test.com</t>
+          <t>https://www.gov.uk/government/people/bim-afolami</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BIMFEEDBACK - BIM Feedback</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>detectado</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>pendiente validación</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://www.gov.uk/hmrc-internal-manuals/business-income-manual/bimfeedback</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Advice Letter: Bim Afolami, Chief of Staff and Strategy, Acrisure, LLC</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>detectado</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>pendiente validación</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://www.gov.uk/government/publications/afolami-bim-economic-secretary-to-the-treasury-acoba-advice/advice-letter-bim-afolami-chief-of-staff-and-strategy-acrisure-llc</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Advice Letter: Bim Afolami, Senior Adviser to the CEO, Peel Hunt</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>detectado</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>pendiente validación</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://www.gov.uk/government/publications/afolami-bim-economic-secretary-to-the-treasury-acoba-advice/advice-letter-bim-afolami-senior-adviser-to-the-ceo-peel-hunt</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Advice Letter: Bim Afolami, Non Executive Director, HSBC UK</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>detectado</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>pendiente validación</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://www.gov.uk/government/publications/afolami-bim-economic-secretary-to-the-treasury-acoba-advice/advice-letter-bim-afolami-non-executive-director-hsbc-uk</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Withdrawal and grandfathering of Extra-Statutory Concession BIM 66301: Sub-postmasters</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>detectado</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>pendiente validación</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://www.gov.uk/government/publications/withdrawal-and-grandfathering-of-extra-statutory-concession-bim-66301-sub-postmasters/withdrawal-and-grandfathering-of-extra-statutory-concession-bim-66301-sub-postmasters</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>HS2 supply chain BIM upskilling study</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>detectado</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>pendiente validación</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://www.gov.uk/government/publications/hs2-supply-chain-bim-upskilling-study</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BIM80635 - Computing the amount to assess: business changes: succession and changes in ownership - partial changes in ownership</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>detectado</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>pendiente validación</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://www.gov.uk/hmrc-internal-manuals/business-income-manual/bim80635</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Withdrawal and grandfathering of Extra-Statutory Concession BIM 66301: Sub-postmasters</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>detectado</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>pendiente validación</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://www.gov.uk/government/publications/withdrawal-and-grandfathering-of-extra-statutory-concession-bim-66301-sub-postmasters</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización BIM Wed Apr  8 22:41:07 UTC 2026
</commit_message>
<xml_diff>
--- a/data/bim_normativas.xlsx
+++ b/data/bim_normativas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,348 +455,6 @@
       <c r="H1" t="inlineStr">
         <is>
           <t>fuente</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Bim Afolami MP</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>UK</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-04-08</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>detectado</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>pendiente validación</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>https://www.gov.uk/government/people/bim-afolami</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>BIMFEEDBACK - BIM Feedback</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>UK</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2026-04-08</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>detectado</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>pendiente validación</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>https://www.gov.uk/hmrc-internal-manuals/business-income-manual/bimfeedback</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Advice Letter: Bim Afolami, Chief of Staff and Strategy, Acrisure, LLC</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>UK</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2026-04-08</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>detectado</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>pendiente validación</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>https://www.gov.uk/government/publications/afolami-bim-economic-secretary-to-the-treasury-acoba-advice/advice-letter-bim-afolami-chief-of-staff-and-strategy-acrisure-llc</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Advice Letter: Bim Afolami, Senior Adviser to the CEO, Peel Hunt</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>UK</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2026-04-08</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>detectado</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>pendiente validación</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>https://www.gov.uk/government/publications/afolami-bim-economic-secretary-to-the-treasury-acoba-advice/advice-letter-bim-afolami-senior-adviser-to-the-ceo-peel-hunt</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Advice Letter: Bim Afolami, Non Executive Director, HSBC UK</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>UK</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>2026-04-08</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>detectado</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>pendiente validación</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>https://www.gov.uk/government/publications/afolami-bim-economic-secretary-to-the-treasury-acoba-advice/advice-letter-bim-afolami-non-executive-director-hsbc-uk</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Withdrawal and grandfathering of Extra-Statutory Concession BIM 66301: Sub-postmasters</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>UK</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>2026-04-08</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>detectado</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>pendiente validación</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>https://www.gov.uk/government/publications/withdrawal-and-grandfathering-of-extra-statutory-concession-bim-66301-sub-postmasters/withdrawal-and-grandfathering-of-extra-statutory-concession-bim-66301-sub-postmasters</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>HS2 supply chain BIM upskilling study</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>UK</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>2026-04-08</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>detectado</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>pendiente validación</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>https://www.gov.uk/government/publications/hs2-supply-chain-bim-upskilling-study</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>BIM80635 - Computing the amount to assess: business changes: succession and changes in ownership - partial changes in ownership</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>UK</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>2026-04-08</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>detectado</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>pendiente validación</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>https://www.gov.uk/hmrc-internal-manuals/business-income-manual/bim80635</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Withdrawal and grandfathering of Extra-Statutory Concession BIM 66301: Sub-postmasters</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>UK</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>2026-04-08</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>detectado</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>pendiente validación</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>https://www.gov.uk/government/publications/withdrawal-and-grandfathering-of-extra-statutory-concession-bim-66301-sub-postmasters</t>
         </is>
       </c>
     </row>

</xml_diff>